<commit_message>
GridTracker güncelleme - 2026-05-18
- todayOverall: 1,320,477.49 → 1,506,005.74 (yeni T2 Overall)
- bist_tracker.html ve data.json güncellendi
- 2.xlsx, ATR_Sonuc.xlsx, Destek_Direc_Seviyeleri.xlsx güncellendi
- Python scriptleri güncellendi

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2.xlsx
+++ b/2.xlsx
@@ -548,7 +548,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>0.45</x:v>
+        <x:v>0.27</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
@@ -559,7 +559,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>1050741.08</x:v>
+        <x:v>390668.18</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
@@ -570,7 +570,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>1047188.16</x:v>
+        <x:v>165155.2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
@@ -581,7 +581,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>391897.49</x:v>
+        <x:v>1340850.54</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
@@ -592,7 +592,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>1432260.9</x:v>
+        <x:v>1500473.81</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
@@ -603,7 +603,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>1437567.57</x:v>
+        <x:v>1503392.72</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
@@ -614,7 +614,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>1439085.65</x:v>
+        <x:v>1506005.74</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:3">
@@ -658,7 +658,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>1047188.16</x:v>
+        <x:v>165155.2</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:3">
@@ -680,7 +680,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>1047188.16</x:v>
+        <x:v>165155.2</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:3">

</xml_diff>